<commit_message>
feat: Add kit contents extraction for component lists
- Extract kit component tables (Q.tà, Descrizione, Codice format)
- Parse quantity, description, and SKU code for each component
- Handle both spec tables and kit contents in extraction

Kit extraction now captures:
- Component SKU codes
- Component descriptions/names
- Quantities

Matching SKUs found in kit files: 6+ components per kit
</commit_message>
<xml_diff>
--- a/output/learning/028_LEADER_kit_PERFECT_60.xlsx
+++ b/output/learning/028_LEADER_kit_PERFECT_60.xlsx
@@ -523,11 +523,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:S8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="43" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
@@ -645,11 +645,207 @@
       </c>
     </row>
     <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>104415</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>A</t>
-        </is>
-      </c>
+          <t>Attuatori 415 230V</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>790077</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Scheda elettronica E045S</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>720119</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Contenitore mod.E per schede elettroniche</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>410029</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Lampeggiatore XLED</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>785103</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Coppia di fotocellule XP20B D</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>787025</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ricevente XF FDS 433-868</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>787017</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Trasmittente 2 canali XT2 FDS 433-868</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>